<commit_message>
updated companies list and reran data pipeline
</commit_message>
<xml_diff>
--- a/data/QPM Student Stock Picks.xlsx
+++ b/data/QPM Student Stock Picks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jason\Documents\FORDHAM MSQF\2026-H2 Quantitative Portfolio Management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hankrugg/Fordham/Fall26/QuantPM/PM/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E9DFDD2-75D3-4F18-93F2-0683BA5322BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A622A6B-E22A-074C-9DBB-A766DC996CA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{B9AC1792-E50D-4783-84C7-4B2A5815088C}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="15500" xr2:uid="{B9AC1792-E50D-4783-84C7-4B2A5815088C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -185,12 +185,6 @@
     <t>DigitalOcean Holdings, Inc.</t>
   </si>
   <si>
-    <t>CRWV</t>
-  </si>
-  <si>
-    <t>CoreWeave, Inc.</t>
-  </si>
-  <si>
     <t>NET</t>
   </si>
   <si>
@@ -233,12 +227,6 @@
     <t>Oruka Therapeutics, Inc.</t>
   </si>
   <si>
-    <t>RDDT</t>
-  </si>
-  <si>
-    <t>Reddit, Inc.</t>
-  </si>
-  <si>
     <t>PG</t>
   </si>
   <si>
@@ -369,6 +357,18 @@
   </si>
   <si>
     <t>Student Name</t>
+  </si>
+  <si>
+    <t>UPST</t>
+  </si>
+  <si>
+    <t>Upstart Holdings Inc.</t>
+  </si>
+  <si>
+    <t>CME</t>
+  </si>
+  <si>
+    <t>CME Group Inc.</t>
   </si>
 </sst>
 </file>
@@ -884,42 +884,42 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10B7C2DB-323F-4283-8608-D74F94E533A6}">
   <dimension ref="A1:F52"/>
-  <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" style="2"/>
-    <col min="2" max="2" width="10.6328125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="36.6328125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="24.6328125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.6328125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.6328125" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="8.6640625" style="2"/>
+    <col min="2" max="2" width="10.6640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="36.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="24.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="6"/>
       <c r="B1" s="6"/>
       <c r="C1" s="19" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D1" s="5"/>
       <c r="E1" s="6"/>
     </row>
-    <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6"/>
       <c r="B2" s="20" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -936,7 +936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -953,7 +953,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -970,7 +970,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -984,7 +984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -998,7 +998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -1015,7 +1015,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -1032,7 +1032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>8</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -1063,7 +1063,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>12</v>
       </c>
@@ -1105,7 +1105,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>14</v>
       </c>
@@ -1133,7 +1133,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>15</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>16</v>
       </c>
@@ -1161,7 +1161,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -1175,7 +1175,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>18</v>
       </c>
@@ -1189,77 +1189,77 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>19</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>49</v>
+        <v>109</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>50</v>
+        <v>110</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>20</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>21</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D23" s="18" t="s">
         <v>7</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>22</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D24" s="18" t="s">
         <v>7</v>
       </c>
       <c r="F24" s="20" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
         <v>23</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>7</v>
@@ -1268,15 +1268,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>24</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>7</v>
@@ -1285,15 +1285,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>25</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>7</v>
@@ -1302,323 +1302,323 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>26</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D28" s="12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>27</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
         <v>28</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
         <v>29</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
         <v>30</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D32" s="12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
         <v>31</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>65</v>
+        <v>107</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>66</v>
+        <v>108</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
         <v>32</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
         <v>33</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
         <v>34</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
         <v>35</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
         <v>36</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D38" s="14" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
         <v>37</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D39" s="12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
         <v>38</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
         <v>39</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
         <v>40</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D42" s="10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
         <v>41</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
         <v>42</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
         <v>43</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
         <v>44</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
         <v>45</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D47" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
         <v>46</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>47</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>48</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>16</v>
@@ -1627,15 +1627,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>49</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>16</v>
@@ -1644,15 +1644,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
         <v>50</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>16</v>

</xml_diff>